<commit_message>
Record research progress and TACCS testing proposals
</commit_message>
<xml_diff>
--- a/Timelog.xlsx
+++ b/Timelog.xlsx
@@ -4,13 +4,11 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matae\OneDrive\Desktop\Coding-Projects\local-play-bootstrap-main\Thesis_ML\"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A0EEC1-F79E-4586-862D-1174B28F316E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2004E26B-F1E0-409D-9467-189499A7AA02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1545" yWindow="4725" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5295" yWindow="3330" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Time Log" sheetId="1" r:id="rId1"/>
@@ -37,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>Thesis ML - Time Log</t>
   </si>
@@ -85,6 +83,21 @@
   </si>
   <si>
     <t>Adding a weekly journal log to my repo and filling it out. Working on cleaning up various things and commiting the working repo tree and pushing to github.</t>
+  </si>
+  <si>
+    <t>Weekly thesis meeting with Dr. Macdonald.</t>
+  </si>
+  <si>
+    <t>Size ablation test nearly through epoch 3 of the 60m model. Looking over and analyzing results; looking for learning trend in loss signals. Decided model training can no longer be done on home computer.</t>
+  </si>
+  <si>
+    <t>Working on writing TACCS usage proposal.</t>
+  </si>
+  <si>
+    <t>Researching how instruction teaching and LLM post-training are done on a more technical level.</t>
+  </si>
+  <si>
+    <t>Looking into getting larger replay dataset of human replays. Confirmed API pathway to accessing Blizzards research dataset of SC2 replay packs.</t>
   </si>
 </sst>
 </file>
@@ -578,14 +591,14 @@
       </c>
       <c r="B2" s="2">
         <f>ROUND(SUM(D5:D304),2)</f>
-        <v>12.25</v>
+        <v>20.25</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="3">
         <f>COUNT(D5:D304)</f>
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>3</v>
@@ -735,64 +748,112 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E12" s="13"/>
+      <c r="A12" s="6">
+        <v>46267</v>
+      </c>
+      <c r="B12" s="11">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C12" s="11">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="D12" s="12">
+        <f t="shared" si="0"/>
+        <v>0.50000000000000089</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="14"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E13" s="17"/>
+      <c r="A13" s="6">
+        <v>46271</v>
+      </c>
+      <c r="B13" s="15">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C13" s="15">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="D13" s="16">
+        <f t="shared" si="0"/>
+        <v>1.5000000000000013</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="10"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E14" s="13"/>
+      <c r="A14" s="6">
+        <v>46274</v>
+      </c>
+      <c r="B14" s="11">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C14" s="11">
+        <v>0.375</v>
+      </c>
+      <c r="D14" s="12">
+        <f t="shared" si="0"/>
+        <v>1.0000000000000004</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E15" s="17"/>
+      <c r="A15" s="6">
+        <v>46276</v>
+      </c>
+      <c r="B15" s="15">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="C15" s="15">
+        <v>0.375</v>
+      </c>
+      <c r="D15" s="16">
+        <f t="shared" si="0"/>
+        <v>1.9999999999999996</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E16" s="13"/>
+      <c r="A16" s="6">
+        <v>46279</v>
+      </c>
+      <c r="B16" s="11">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="C16" s="11">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="D16" s="12">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="14"/>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E17" s="17"/>
+      <c r="A17" s="6">
+        <v>46280</v>
+      </c>
+      <c r="B17" s="15">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="C17" s="15">
+        <v>0.48958333333333331</v>
+      </c>
+      <c r="D17" s="16">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="10"/>

</xml_diff>

<commit_message>
Record AR-arm decision in research journal and time log
Logs the 9/14-9/20 decision to build an autoregressive training pipeline in
TensorFlow as the experimental study arm for comparison against the diffusion
model, plus early thinking on unconditioned pre-training for that arm.
</commit_message>
<xml_diff>
--- a/Timelog.xlsx
+++ b/Timelog.xlsx
@@ -4,9 +4,11 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15"/>
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matae\OneDrive\Desktop\Coding-Projects\local-play-bootstrap-main\Thesis_ML\"/>
+    </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2004E26B-F1E0-409D-9467-189499A7AA02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C70C10-7F33-490E-B322-7FF9027BC519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5295" yWindow="3330" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>Thesis ML - Time Log</t>
   </si>
@@ -98,6 +100,9 @@
   </si>
   <si>
     <t>Looking into getting larger replay dataset of human replays. Confirmed API pathway to accessing Blizzards research dataset of SC2 replay packs.</t>
+  </si>
+  <si>
+    <t>Beginning working on the BPE tokenizer and architecting out the AR model experimental test pipeline.</t>
   </si>
 </sst>
 </file>
@@ -591,14 +596,14 @@
       </c>
       <c r="B2" s="2">
         <f>ROUND(SUM(D5:D304),2)</f>
-        <v>20.25</v>
+        <v>22.25</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="3">
         <f>COUNT(D5:D304)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>3</v>
@@ -856,14 +861,22 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E18" s="13"/>
+      <c r="A18" s="6">
+        <v>46285</v>
+      </c>
+      <c r="B18" s="11">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="C18" s="11">
+        <v>0.375</v>
+      </c>
+      <c r="D18" s="12">
+        <f t="shared" si="0"/>
+        <v>1.9999999999999996</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>

</xml_diff>

<commit_message>
Add joint sequence and BPE inspection preview
</commit_message>
<xml_diff>
--- a/Timelog.xlsx
+++ b/Timelog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matae\OneDrive\Desktop\Coding-Projects\local-play-bootstrap-main\Thesis_ML\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C70C10-7F33-490E-B322-7FF9027BC519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF8BC7E1-49F7-4CC2-A5C9-7E2DE4AB9B8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5295" yWindow="3330" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Thesis ML - Time Log</t>
   </si>
@@ -103,6 +103,15 @@
   </si>
   <si>
     <t>Beginning working on the BPE tokenizer and architecting out the AR model experimental test pipeline.</t>
+  </si>
+  <si>
+    <t>Working out conceptualizing non-conditioned pre-training; particularly how to present both players sequences in generated sequence.</t>
+  </si>
+  <si>
+    <t>Working with coding agent to begin building out the new sequence presentation and begin building out tokenization on top of it.</t>
+  </si>
+  <si>
+    <t>Working on tweaking the BPE tokenizer. Nailing down the merging stop point. Tidying up the human facing decoding of tokenized windows.</t>
   </si>
 </sst>
 </file>
@@ -596,14 +605,14 @@
       </c>
       <c r="B2" s="2">
         <f>ROUND(SUM(D5:D304),2)</f>
-        <v>22.25</v>
+        <v>26.75</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="3">
         <f>COUNT(D5:D304)</f>
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>3</v>
@@ -879,34 +888,58 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="14"/>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E19" s="17"/>
+      <c r="A19" s="6">
+        <v>46285</v>
+      </c>
+      <c r="B19" s="15">
+        <v>0.40625</v>
+      </c>
+      <c r="C19" s="15">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="D19" s="16">
+        <f t="shared" si="0"/>
+        <v>0.49999999999999956</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E20" s="13"/>
+      <c r="A20" s="6">
+        <v>46285</v>
+      </c>
+      <c r="B20" s="15">
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="C20" s="11">
+        <v>0.63541666666666663</v>
+      </c>
+      <c r="D20" s="12">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="14"/>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="E21" s="17"/>
+      <c r="A21" s="6">
+        <v>46286</v>
+      </c>
+      <c r="B21" s="15">
+        <v>0.6875</v>
+      </c>
+      <c r="C21" s="15">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="D21" s="16">
+        <f t="shared" si="0"/>
+        <v>0.99999999999999911</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="10"/>

</xml_diff>